<commit_message>
Add desktop QR code
</commit_message>
<xml_diff>
--- a/人員資料.xlsx
+++ b/人員資料.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zheng\Desktop\專師排班\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596A506C-F73C-49BB-A5DF-0A5AE6A0084C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C20FBB-419A-4D2F-A8DD-0DF54F0A3C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{48D69275-A82C-4262-BE18-50E54801D2B4}"/>
+    <workbookView xWindow="4760" yWindow="920" windowWidth="14400" windowHeight="8170" xr2:uid="{48D69275-A82C-4262-BE18-50E54801D2B4}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -69,9 +69,6 @@
     <t>沈宛君</t>
   </si>
   <si>
-    <t>張婷婷</t>
-  </si>
-  <si>
     <t>鄭鈺芬</t>
   </si>
   <si>
@@ -171,6 +168,10 @@
   </si>
   <si>
     <t>醫師電話</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>張婷亭</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -600,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
-        <v>14</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F1" s="1"/>
     </row>
@@ -618,7 +619,7 @@
         <v>8064</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2" s="3">
         <v>6231</v>
@@ -633,7 +634,7 @@
         <v>8061</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3">
         <v>5331</v>
@@ -648,7 +649,7 @@
         <v>8287</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="3">
         <v>5619</v>
@@ -663,7 +664,7 @@
         <v>8073</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" s="3">
         <v>6017</v>
@@ -678,14 +679,14 @@
         <v>8049</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3">
         <v>6623</v>
       </c>
       <c r="F6" s="2"/>
       <c r="K6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -696,7 +697,7 @@
         <v>8121</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="3">
         <v>3544</v>
@@ -711,7 +712,7 @@
         <v>8281</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="3">
         <v>3652</v>
@@ -726,7 +727,7 @@
         <v>8122</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9" s="3">
         <v>5520</v>
@@ -735,13 +736,13 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="B10">
         <v>8132</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="3">
         <v>8048</v>
@@ -750,13 +751,13 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>8152</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="3">
         <v>5318</v>
@@ -765,13 +766,13 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>8173</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="3">
         <v>8002</v>
@@ -780,13 +781,13 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13">
         <v>8417</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E13" s="3">
         <v>6654</v>
@@ -795,7 +796,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="D14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="3">
         <v>5189</v>
@@ -804,7 +805,7 @@
     </row>
     <row r="15" spans="1:11">
       <c r="D15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="3">
         <v>8024</v>
@@ -813,7 +814,7 @@
     </row>
     <row r="16" spans="1:11">
       <c r="D16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16" s="3">
         <v>6077</v>
@@ -822,7 +823,7 @@
     </row>
     <row r="17" spans="4:6">
       <c r="D17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E17" s="3">
         <v>6181</v>
@@ -831,14 +832,14 @@
     </row>
     <row r="18" spans="4:6">
       <c r="D18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="4:6">
       <c r="D19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E19" s="3">
         <v>8246</v>
@@ -847,7 +848,7 @@
     </row>
     <row r="20" spans="4:6">
       <c r="D20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="3">
         <v>5768</v>
@@ -856,7 +857,7 @@
     </row>
     <row r="21" spans="4:6">
       <c r="D21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E21" s="3">
         <v>6482</v>
@@ -865,14 +866,14 @@
     </row>
     <row r="22" spans="4:6">
       <c r="D22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="4:6">
       <c r="D23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E23" s="3">
         <v>3354</v>
@@ -881,25 +882,25 @@
     </row>
     <row r="24" spans="4:6">
       <c r="D24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="4:6">
       <c r="D25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="4:6">
       <c r="D26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F26" s="2"/>
     </row>
     <row r="27" spans="4:6">
       <c r="D27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F27" s="2"/>
     </row>

</xml_diff>